<commit_message>
changes in import excel and other improvements
</commit_message>
<xml_diff>
--- a/public/resources/template_import_excel_topics_and_activities.xlsx
+++ b/public/resources/template_import_excel_topics_and_activities.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27830"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28324"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC IJO\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Internship Vannes Theo S\sangnila-lms\public\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF1DCFE5-E5BA-4D12-9CB3-4D0F874C4D56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C257F016-9BD6-4021-835A-3945522C40DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3930" yWindow="1575" windowWidth="21600" windowHeight="13920" xr2:uid="{36DCB5BE-75A0-421E-9C01-C78017D39B37}"/>
+    <workbookView xWindow="1515" yWindow="1515" windowWidth="21600" windowHeight="11385" xr2:uid="{36DCB5BE-75A0-421E-9C01-C78017D39B37}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,18 +25,21 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
   <si>
     <t>topic</t>
-  </si>
-  <si>
-    <t>material</t>
   </si>
   <si>
     <t>description</t>
   </si>
   <si>
     <t>link</t>
+  </si>
+  <si>
+    <t>session</t>
+  </si>
+  <si>
+    <t>activity</t>
   </si>
 </sst>
 </file>
@@ -134,9 +137,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -174,7 +177,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -280,7 +283,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -422,7 +425,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -430,82 +433,94 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{89D30DA1-E9EE-4DE0-8C35-496265AD309C}">
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="31" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.85546875" customWidth="1"/>
     <col min="2" max="2" width="41.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="74" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="23.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="49.42578125" customWidth="1"/>
+    <col min="4" max="4" width="52.85546875" customWidth="1"/>
+    <col min="5" max="5" width="29.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="C1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="E1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="1"/>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
-      <c r="D2" s="2"/>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D2" s="1"/>
+      <c r="E2" s="2"/>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
-      <c r="D3" s="2"/>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D3" s="1"/>
+      <c r="E3" s="2"/>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
       <c r="B4" s="1"/>
       <c r="C4" s="1"/>
-      <c r="D4" s="2"/>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D4" s="1"/>
+      <c r="E4" s="2"/>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
       <c r="B5" s="1"/>
       <c r="C5" s="1"/>
-      <c r="D5" s="2"/>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D5" s="1"/>
+      <c r="E5" s="2"/>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
       <c r="B6" s="1"/>
       <c r="C6" s="1"/>
-      <c r="D6" s="2"/>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D6" s="1"/>
+      <c r="E6" s="2"/>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
       <c r="B7" s="1"/>
       <c r="C7" s="1"/>
-      <c r="D7" s="2"/>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D7" s="1"/>
+      <c r="E7" s="2"/>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="1"/>
       <c r="B8" s="1"/>
       <c r="C8" s="1"/>
-      <c r="D8" s="2"/>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D8" s="1"/>
+      <c r="E8" s="2"/>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="1"/>
       <c r="B9" s="1"/>
       <c r="C9" s="1"/>
       <c r="D9" s="1"/>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E9" s="1"/>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="1"/>
       <c r="B10" s="1"/>
       <c r="C10" s="1"/>
       <c r="D10" s="1"/>
+      <c r="E10" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>